<commit_message>
refactor(feedback): replace RepeatCount with Index in JourneyFeedbackStep and related components
</commit_message>
<xml_diff>
--- a/docs/Journey-Editor.xlsx
+++ b/docs/Journey-Editor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repo\ahuelsmann\MOBAflow\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86BB70FC-C624-4086-A9A8-E4B18F619D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D800EC-6EB5-4212-9574-5DF00DB3FF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{46B0417C-9ABD-4968-BA3B-6464BB1A6AE6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="20">
   <si>
     <t>Journey</t>
   </si>
@@ -53,15 +53,6 @@
     <t>Switch Next Station</t>
   </si>
   <si>
-    <t>Count</t>
-  </si>
-  <si>
-    <t>RE1</t>
-  </si>
-  <si>
-    <t>Westfalen-Express</t>
-  </si>
-  <si>
     <t>Workflow</t>
   </si>
   <si>
@@ -75,6 +66,39 @@
   </si>
   <si>
     <t>Workflow1</t>
+  </si>
+  <si>
+    <t>Bielefeld</t>
+  </si>
+  <si>
+    <t>Herford</t>
+  </si>
+  <si>
+    <t>Minden</t>
+  </si>
+  <si>
+    <t>Stations</t>
+  </si>
+  <si>
+    <t>JourneyManager</t>
+  </si>
+  <si>
+    <t>FeedbackSequence</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>…</t>
+  </si>
+  <si>
+    <t>CurrentIndex</t>
+  </si>
+  <si>
+    <t>CurrentStation</t>
   </si>
 </sst>
 </file>
@@ -126,13 +150,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -467,112 +497,208 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874AB08F-7AB9-403F-9B25-88C01D634932}">
-  <dimension ref="A2:F13"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="5.53125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.9296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.9296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="3" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="6" max="8" width="26.6640625" customWidth="1"/>
+    <col min="9" max="9" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="D4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.45"/>
-    <row r="4" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="2" t="s">
+      <c r="H4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D6" s="3">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D7" s="3">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D8" s="3">
         <v>4</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D9" s="3">
+        <v>5</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D10" s="3">
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" t="s">
+        <v>2</v>
+      </c>
+      <c r="H10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D11" s="3">
         <v>7</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E11" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D12" s="3">
         <v>8</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>3</v>
+      </c>
+      <c r="G12" t="s">
+        <v>2</v>
+      </c>
+      <c r="H12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="C14" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D15" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D16" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C18" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="D19" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="D20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="1" t="s">
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="D21" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B5">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="D22" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C24" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="D25" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="D26" s="5" t="s">
         <v>1</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B7">
-        <v>3</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B8">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B10">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B11">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B12">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B13">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>